<commit_message>
Add regression utility-gap tables and updated classification analysis outputs.
</commit_message>
<xml_diff>
--- a/Agreed analysis/classification/classification_utility_gap_cd_analysis.xlsx
+++ b/Agreed analysis/classification/classification_utility_gap_cd_analysis.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accuracy_Nemenyi_Sig" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precision_Nemenyi_Sig" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recall_Nemenyi_Sig" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F1_Nemenyi_Sig" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,7 +644,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>accuracy_gap_critical_difference_diagram.png</t>
+          <t>accuracy_gap_critical_difference_diagram.png/.svg</t>
         </is>
       </c>
     </row>
@@ -699,7 +700,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>precision_gap_critical_difference_diagram.png</t>
+          <t>precision_gap_critical_difference_diagram.png/.svg</t>
         </is>
       </c>
     </row>
@@ -755,7 +756,63 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>recall_gap_critical_difference_diagram.png</t>
+          <t>recall_gap_critical_difference_diagram.png/.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>F1_Gap</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>31.18518518518516</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.746949162351424e-05</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ForestDiffusion</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>TabDDPM</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>6.888888888888889</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>f1_gap_analysis.xlsx</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>f1_gap_critical_difference_diagram.png/.svg</t>
         </is>
       </c>
     </row>
@@ -770,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,6 +851,11 @@
           <t>Recall</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -810,6 +872,9 @@
       <c r="D2" t="n">
         <v>2.1111</v>
       </c>
+      <c r="E2" t="n">
+        <v>1.3333</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -826,6 +891,9 @@
       <c r="D3" t="n">
         <v>4.4444</v>
       </c>
+      <c r="E3" t="n">
+        <v>3.8889</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -842,6 +910,9 @@
       <c r="D4" t="n">
         <v>3.8889</v>
       </c>
+      <c r="E4" t="n">
+        <v>3.4444</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -858,6 +929,9 @@
       <c r="D5" t="n">
         <v>4.1111</v>
       </c>
+      <c r="E5" t="n">
+        <v>4.2222</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -874,37 +948,46 @@
       <c r="D6" t="n">
         <v>4.4444</v>
       </c>
+      <c r="E6" t="n">
+        <v>5.1111</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5.7778</v>
+        <v>6.3333</v>
       </c>
       <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
         <v>5.1111</v>
       </c>
-      <c r="D7" t="n">
-        <v>6.1111</v>
+      <c r="E7" t="n">
+        <v>4.8889</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.3333</v>
+        <v>5.7778</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>5.1111</v>
       </c>
       <c r="D8" t="n">
-        <v>5.1111</v>
+        <v>6.1111</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6.2222</v>
       </c>
     </row>
     <row r="9">
@@ -921,6 +1004,9 @@
       </c>
       <c r="D9" t="n">
         <v>5.7778</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.8889</v>
       </c>
     </row>
   </sheetData>
@@ -1328,4 +1414,146 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Generator_A</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Generator_B</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AvgRank_A</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>AvgRank_B</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p_value</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Significant_alpha_0.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ForestDiffusion</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TabDDPM</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.888888888888889</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4.104257745418671e-05</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ForestDiffusion</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CTGAN</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6.222222222222222</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0006060957281330825</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ForestDiffusion</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GaussianCopula</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5.111111111111111</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.02377669007998073</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ForestDiffusion</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CopulaGAN</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4.888888888888889</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.04333096070012921</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>